<commit_message>
Add files for tests for 2026.1
</commit_message>
<xml_diff>
--- a/metamodel_py/tests/qs1_files/Data/inputs/Model_Parameters.xlsx
+++ b/metamodel_py/tests/qs1_files/Data/inputs/Model_Parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\RDR\metamodel_py\tests\qs1_files\Data\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ACB68E6-2870-455B-93FE-1AAA3C4934E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78CB0C80-AB55-4DD4-922B-032DAD4ABFF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="7" r:id="rId1"/>
@@ -72,9 +72,6 @@
   </si>
   <si>
     <t>HazardDim2</t>
-  </si>
-  <si>
-    <t>base</t>
   </si>
   <si>
     <t>02</t>
@@ -277,6 +274,9 @@
   </si>
   <si>
     <t>Enter one or more number(s) defining how the probability of all hazard event(s) will increase or decrease year-on-year throughout the analysis period. A value of 1 means no change across years in hazard event probability values; a value above 1 means an increase in frequency over time; a value below 1 means a decrease in frequency over time.</t>
+  </si>
+  <si>
+    <t>standard</t>
   </si>
 </sst>
 </file>
@@ -738,13 +738,13 @@
   <dimension ref="A1:J31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="120.6640625" style="18" customWidth="1"/>
+    <col min="1" max="1" width="120.77734375" style="18" customWidth="1"/>
     <col min="2" max="2" width="42.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" s="6" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -770,7 +770,7 @@
     </row>
     <row r="3" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="7"/>
@@ -796,7 +796,7 @@
     </row>
     <row r="5" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B5" s="7"/>
       <c r="C5" s="7"/>
@@ -810,7 +810,7 @@
     </row>
     <row r="6" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B6" s="7"/>
       <c r="C6" s="7"/>
@@ -836,7 +836,7 @@
     </row>
     <row r="8" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B8" s="7"/>
       <c r="C8" s="7"/>
@@ -850,7 +850,7 @@
     </row>
     <row r="9" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
@@ -876,7 +876,7 @@
     </row>
     <row r="11" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B11" s="7"/>
       <c r="C11" s="7"/>
@@ -890,7 +890,7 @@
     </row>
     <row r="12" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A12" s="13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B12" s="7"/>
       <c r="C12" s="7"/>
@@ -916,7 +916,7 @@
     </row>
     <row r="14" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A14" s="15" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B14" s="7"/>
       <c r="C14" s="7"/>
@@ -930,7 +930,7 @@
     </row>
     <row r="15" spans="1:10" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
@@ -956,7 +956,7 @@
     </row>
     <row r="17" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A17" s="15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
@@ -970,7 +970,7 @@
     </row>
     <row r="18" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
@@ -996,7 +996,7 @@
     </row>
     <row r="20" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" s="15" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
@@ -1010,7 +1010,7 @@
     </row>
     <row r="21" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A21" s="18" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B21" s="7"/>
       <c r="C21" s="7"/>
@@ -1152,7 +1152,7 @@
   <dimension ref="A1:B18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.33203125" customWidth="1"/>
+    <col min="1" max="1" width="19.21875" customWidth="1"/>
     <col min="2" max="2" width="13.44140625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1164,7 +1164,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="B2" s="2"/>
     </row>
@@ -1227,7 +1227,7 @@
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1247,11 +1247,11 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.44140625" customWidth="1"/>
-    <col min="2" max="2" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1259,31 +1259,31 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -1295,17 +1295,14 @@
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" s="2"/>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="2"/>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="2"/>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1318,11 +1315,11 @@
   <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.109375" customWidth="1"/>
+    <col min="1" max="1" width="14.21875" customWidth="1"/>
     <col min="2" max="2" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="39.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="39.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.21875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7.5546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1349,10 +1346,10 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C2">
         <v>10</v>
@@ -1361,7 +1358,7 @@
         <v>0</v>
       </c>
       <c r="E2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F2">
         <v>0.1</v>
@@ -1369,10 +1366,10 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -1381,7 +1378,7 @@
         <v>0</v>
       </c>
       <c r="E3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F3">
         <v>0.9</v>
@@ -1425,12 +1422,12 @@
   <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">

</xml_diff>